<commit_message>
new AMR devices installed on floor 1 and positions adjusted
</commit_message>
<xml_diff>
--- a/Summer_Ridge_Master_Sheet.xlsx
+++ b/Summer_Ridge_Master_Sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Summer Ridge/Estate Management/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="136" documentId="8_{61B75D5B-E2B9-4A15-B62A-CAAC6678E594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A28AD59-97CB-4F70-8687-EDD74F94C192}"/>
+  <xr:revisionPtr revIDLastSave="154" documentId="8_{61B75D5B-E2B9-4A15-B62A-CAAC6678E594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C89DEF5B-AEEC-48BA-ADBE-176A3AA6FF97}"/>
   <bookViews>
-    <workbookView xWindow="71880" yWindow="-1530" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{97778EF9-769A-4231-8D2B-397889BE3400}"/>
+    <workbookView xWindow="43080" yWindow="-7455" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{97778EF9-769A-4231-8D2B-397889BE3400}"/>
   </bookViews>
   <sheets>
     <sheet name="Elec" sheetId="1" r:id="rId1"/>
@@ -988,7 +988,8 @@
     <col min="1" max="1" width="17.73046875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.86328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.86328125" customWidth="1"/>
-    <col min="4" max="4" width="17.3984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.19921875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
@@ -3722,8 +3723,8 @@
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="8.1328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.73046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.59765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.45">
@@ -3745,7 +3746,7 @@
         <v>25003273</v>
       </c>
       <c r="C2" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
@@ -3756,7 +3757,7 @@
         <v>25003187</v>
       </c>
       <c r="C3" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
@@ -3789,7 +3790,7 @@
         <v>25003302</v>
       </c>
       <c r="C6" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.45">
@@ -3811,7 +3812,7 @@
         <v>25003167</v>
       </c>
       <c r="C8" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
@@ -3844,7 +3845,7 @@
         <v>25003183</v>
       </c>
       <c r="C11" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.45">
@@ -3877,7 +3878,7 @@
         <v>25003188</v>
       </c>
       <c r="C14" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.45">
@@ -3888,7 +3889,7 @@
         <v>25003184</v>
       </c>
       <c r="C15" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.45">
@@ -3899,7 +3900,7 @@
         <v>25003218</v>
       </c>
       <c r="C16" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.45">
@@ -3910,7 +3911,7 @@
         <v>25003212</v>
       </c>
       <c r="C17" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.45">
@@ -3921,7 +3922,7 @@
         <v>25003164</v>
       </c>
       <c r="C18" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.45">
@@ -3932,7 +3933,7 @@
         <v>25003197</v>
       </c>
       <c r="C19" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.45">
@@ -3954,7 +3955,7 @@
         <v>25000769</v>
       </c>
       <c r="C21" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.45">
@@ -4009,7 +4010,7 @@
         <v>25003228</v>
       </c>
       <c r="C26" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.45">
@@ -4053,7 +4054,7 @@
         <v>25003225</v>
       </c>
       <c r="C30" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.45">

</xml_diff>